<commit_message>
Check-list formation : synthèse par module et acteur corrigée
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XGyegFqNtRrxVgA5XBt8RL
</commit_message>
<xml_diff>
--- a/docs/checklist-fin-formation.xlsx
+++ b/docs/checklist-fin-formation.xlsx
@@ -2929,7 +2929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2986,7 +2986,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Créer, confirmer et importer une commande</t>
+          <t>Responsable commercial</t>
         </is>
       </c>
       <c r="C2" s="5">
@@ -3018,7 +3018,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Gérer clients et vendeurs partenaires (fiche, candidature)</t>
+          <t>Client</t>
         </is>
       </c>
       <c r="C3" s="5">
@@ -3050,7 +3050,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Établir facture, reçu, avoir</t>
+          <t>Préparateur</t>
         </is>
       </c>
       <c r="C4" s="5">
@@ -3082,7 +3082,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Programmer une livraison depuis le portail</t>
+          <t>Superviseur des livraisons</t>
         </is>
       </c>
       <c r="C5" s="5">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Suivre sa livraison et signer la réception</t>
+          <t>Livreur</t>
         </is>
       </c>
       <c r="C6" s="5">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Préparer commande, imprimer étiquettes colis</t>
+          <t>Vendeur partenaire</t>
         </is>
       </c>
       <c r="C7" s="5">
@@ -3178,7 +3178,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Réceptionner collectes et retours de colis</t>
+          <t>Caissier</t>
         </is>
       </c>
       <c r="C8" s="5">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Saisir entrées de stock et inventaire</t>
+          <t>Direction générale</t>
         </is>
       </c>
       <c r="C9" s="5">
@@ -3242,7 +3242,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Créer produits, traiter candidatures vendeurs</t>
+          <t>Administrateur</t>
         </is>
       </c>
       <c r="C10" s="5">
@@ -3269,12 +3269,12 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Livraison (Distributions)</t>
+          <t>Gestion de taxi (Transport)</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Affecter livreur, planifier collecte, suivre course</t>
+          <t>Gestionnaire de flotte</t>
         </is>
       </c>
       <c r="C11" s="5">
@@ -3301,12 +3301,12 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Livraison (Distributions)</t>
+          <t>Gestion de taxi (Transport)</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Utiliser tour de contrôle et carte en direct</t>
+          <t>Directeur / propriétaire</t>
         </is>
       </c>
       <c r="C12" s="5">
@@ -3333,12 +3333,12 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Livraison (Distributions)</t>
+          <t>Gestion de taxi (Transport)</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Traiter échecs, retours, incidents</t>
+          <t>Caissier</t>
         </is>
       </c>
       <c r="C13" s="5">
@@ -3365,12 +3365,12 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Livraison (Distributions)</t>
+          <t>Gestion de taxi (Transport)</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Recevoir et traiter une alerte SOS</t>
+          <t>Contrôleur</t>
         </is>
       </c>
       <c r="C14" s="5">
@@ -3397,12 +3397,12 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Livraison (Distributions)</t>
+          <t>Gestion de taxi (Transport)</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Clôturer la journée du centre</t>
+          <t>Comptable</t>
         </is>
       </c>
       <c r="C15" s="5">
@@ -3429,12 +3429,12 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Livraison (Distributions)</t>
+          <t>Gestion de taxi (Transport)</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Gérer livreurs, motos, équipements, maintenance</t>
+          <t>Chauffeur taxi</t>
         </is>
       </c>
       <c r="C16" s="5">
@@ -3461,12 +3461,12 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Livraison (Distributions)</t>
+          <t>Gestion de taxi (Transport)</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Installer l'application et se connecter</t>
+          <t>Administrateur général</t>
         </is>
       </c>
       <c r="C17" s="5">
@@ -3493,12 +3493,12 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Livraison (Distributions)</t>
+          <t>Transversal (Groupe)</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Accepter une mission, statuts de la course</t>
+          <t>Administrateur</t>
         </is>
       </c>
       <c r="C18" s="5">
@@ -3525,12 +3525,12 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Livraison (Distributions)</t>
+          <t>Transversal (Groupe)</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Appeler le client, partager sa position</t>
+          <t>Direction générale</t>
         </is>
       </c>
       <c r="C19" s="5">
@@ -3557,12 +3557,12 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Livraison (Distributions)</t>
+          <t>Transversal (Groupe)</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Obtenir signature et photo de preuve</t>
+          <t>Tous</t>
         </is>
       </c>
       <c r="C20" s="5">
@@ -3583,1574 +3583,6 @@
       </c>
       <c r="G20" s="6">
         <f>IF(C20=0,0,D20/C20)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Livraison (Distributions)</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>Déclarer échec ou retour avec motif</t>
-        </is>
-      </c>
-      <c r="C21" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A21,Checklist!$D$4:$D$71,$B21)</f>
-        <v/>
-      </c>
-      <c r="D21" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A21,Checklist!$D$4:$D$71,$B21,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E21" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A21,Checklist!$D$4:$D$71,$B21,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F21" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A21,Checklist!$D$4:$D$71,$B21,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G21" s="6">
-        <f>IF(C21=0,0,D21/C21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Livraison (Distributions)</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Encaisser contre-remboursement et verser</t>
-        </is>
-      </c>
-      <c r="C22" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A22,Checklist!$D$4:$D$71,$B22)</f>
-        <v/>
-      </c>
-      <c r="D22" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A22,Checklist!$D$4:$D$71,$B22,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E22" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A22,Checklist!$D$4:$D$71,$B22,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F22" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A22,Checklist!$D$4:$D$71,$B22,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G22" s="6">
-        <f>IF(C22=0,0,D22/C22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Livraison (Distributions)</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>Déclencher SOS en cas de danger</t>
-        </is>
-      </c>
-      <c r="C23" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A23,Checklist!$D$4:$D$71,$B23)</f>
-        <v/>
-      </c>
-      <c r="D23" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A23,Checklist!$D$4:$D$71,$B23,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E23" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A23,Checklist!$D$4:$D$71,$B23,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F23" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A23,Checklist!$D$4:$D$71,$B23,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G23" s="6">
-        <f>IF(C23=0,0,D23/C23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Livraison (Distributions)</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Travailler hors ligne puis resynchroniser</t>
-        </is>
-      </c>
-      <c r="C24" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A24,Checklist!$D$4:$D$71,$B24)</f>
-        <v/>
-      </c>
-      <c r="D24" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A24,Checklist!$D$4:$D$71,$B24,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E24" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A24,Checklist!$D$4:$D$71,$B24,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F24" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A24,Checklist!$D$4:$D$71,$B24,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G24" s="6">
-        <f>IF(C24=0,0,D24/C24)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Livraison (Distributions)</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>Publier produits et saisir commandes</t>
-        </is>
-      </c>
-      <c r="C25" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A25,Checklist!$D$4:$D$71,$B25)</f>
-        <v/>
-      </c>
-      <c r="D25" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A25,Checklist!$D$4:$D$71,$B25,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E25" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A25,Checklist!$D$4:$D$71,$B25,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F25" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A25,Checklist!$D$4:$D$71,$B25,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G25" s="6">
-        <f>IF(C25=0,0,D25/C25)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>Livraison (Distributions)</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>Imprimer étiquettes et suivre ses colis</t>
-        </is>
-      </c>
-      <c r="C26" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A26,Checklist!$D$4:$D$71,$B26)</f>
-        <v/>
-      </c>
-      <c r="D26" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A26,Checklist!$D$4:$D$71,$B26,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E26" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A26,Checklist!$D$4:$D$71,$B26,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F26" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A26,Checklist!$D$4:$D$71,$B26,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G26" s="6">
-        <f>IF(C26=0,0,D26/C26)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>Livraison (Distributions)</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Consulter son état et ses versements</t>
-        </is>
-      </c>
-      <c r="C27" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A27,Checklist!$D$4:$D$71,$B27)</f>
-        <v/>
-      </c>
-      <c r="D27" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A27,Checklist!$D$4:$D$71,$B27,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E27" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A27,Checklist!$D$4:$D$71,$B27,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F27" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A27,Checklist!$D$4:$D$71,$B27,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G27" s="6">
-        <f>IF(C27=0,0,D27/C27)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>Livraison (Distributions)</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>Ouvrir et clôturer la caisse, gérer écart</t>
-        </is>
-      </c>
-      <c r="C28" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A28,Checklist!$D$4:$D$71,$B28)</f>
-        <v/>
-      </c>
-      <c r="D28" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A28,Checklist!$D$4:$D$71,$B28,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E28" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A28,Checklist!$D$4:$D$71,$B28,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F28" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A28,Checklist!$D$4:$D$71,$B28,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G28" s="6">
-        <f>IF(C28=0,0,D28/C28)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>Livraison (Distributions)</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>Valider versements livreurs, reverser vendeurs</t>
-        </is>
-      </c>
-      <c r="C29" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A29,Checklist!$D$4:$D$71,$B29)</f>
-        <v/>
-      </c>
-      <c r="D29" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A29,Checklist!$D$4:$D$71,$B29,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E29" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A29,Checklist!$D$4:$D$71,$B29,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F29" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A29,Checklist!$D$4:$D$71,$B29,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G29" s="6">
-        <f>IF(C29=0,0,D29/C29)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>Livraison (Distributions)</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>Accepter ou refuser un écart de caisse</t>
-        </is>
-      </c>
-      <c r="C30" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A30,Checklist!$D$4:$D$71,$B30)</f>
-        <v/>
-      </c>
-      <c r="D30" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A30,Checklist!$D$4:$D$71,$B30,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E30" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A30,Checklist!$D$4:$D$71,$B30,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F30" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A30,Checklist!$D$4:$D$71,$B30,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G30" s="6">
-        <f>IF(C30=0,0,D30/C30)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>Livraison (Distributions)</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>Valider mouvements de caisse et opérations RH</t>
-        </is>
-      </c>
-      <c r="C31" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A31,Checklist!$D$4:$D$71,$B31)</f>
-        <v/>
-      </c>
-      <c r="D31" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A31,Checklist!$D$4:$D$71,$B31,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E31" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A31,Checklist!$D$4:$D$71,$B31,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F31" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A31,Checklist!$D$4:$D$71,$B31,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G31" s="6">
-        <f>IF(C31=0,0,D31/C31)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>Livraison (Distributions)</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>Lire tableau de bord, états, trésorerie</t>
-        </is>
-      </c>
-      <c r="C32" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A32,Checklist!$D$4:$D$71,$B32)</f>
-        <v/>
-      </c>
-      <c r="D32" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A32,Checklist!$D$4:$D$71,$B32,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E32" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A32,Checklist!$D$4:$D$71,$B32,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F32" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A32,Checklist!$D$4:$D$71,$B32,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G32" s="6">
-        <f>IF(C32=0,0,D32/C32)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>Livraison (Distributions)</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>Créer utilisateurs, rôles et droits</t>
-        </is>
-      </c>
-      <c r="C33" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A33,Checklist!$D$4:$D$71,$B33)</f>
-        <v/>
-      </c>
-      <c r="D33" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A33,Checklist!$D$4:$D$71,$B33,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E33" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A33,Checklist!$D$4:$D$71,$B33,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F33" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A33,Checklist!$D$4:$D$71,$B33,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G33" s="6">
-        <f>IF(C33=0,0,D33/C33)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
-        <is>
-          <t>Livraison (Distributions)</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>Lire journal d'audit</t>
-        </is>
-      </c>
-      <c r="C34" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A34,Checklist!$D$4:$D$71,$B34)</f>
-        <v/>
-      </c>
-      <c r="D34" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A34,Checklist!$D$4:$D$71,$B34,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E34" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A34,Checklist!$D$4:$D$71,$B34,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F34" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A34,Checklist!$D$4:$D$71,$B34,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G34" s="6">
-        <f>IF(C34=0,0,D34/C34)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>Livraison (Distributions)</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>Passer en production (vider données d'exercice)</t>
-        </is>
-      </c>
-      <c r="C35" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A35,Checklist!$D$4:$D$71,$B35)</f>
-        <v/>
-      </c>
-      <c r="D35" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A35,Checklist!$D$4:$D$71,$B35,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E35" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A35,Checklist!$D$4:$D$71,$B35,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F35" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A35,Checklist!$D$4:$D$71,$B35,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G35" s="6">
-        <f>IF(C35=0,0,D35/C35)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>Créer véhicule + documents (carte grise, assurance, visite, carte de transport)</t>
-        </is>
-      </c>
-      <c r="C36" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A36,Checklist!$D$4:$D$71,$B36)</f>
-        <v/>
-      </c>
-      <c r="D36" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A36,Checklist!$D$4:$D$71,$B36,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E36" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A36,Checklist!$D$4:$D$71,$B36,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F36" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A36,Checklist!$D$4:$D$71,$B36,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G36" s="6">
-        <f>IF(C36=0,0,D36/C36)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>Gérer statuts, sortie du parc, historique</t>
-        </is>
-      </c>
-      <c r="C37" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A37,Checklist!$D$4:$D$71,$B37)</f>
-        <v/>
-      </c>
-      <c r="D37" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A37,Checklist!$D$4:$D$71,$B37,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E37" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A37,Checklist!$D$4:$D$71,$B37,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F37" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A37,Checklist!$D$4:$D$71,$B37,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G37" s="6">
-        <f>IF(C37=0,0,D37/C37)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>Créer chauffeur + dossier (photo, permis, CNI)</t>
-        </is>
-      </c>
-      <c r="C38" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A38,Checklist!$D$4:$D$71,$B38)</f>
-        <v/>
-      </c>
-      <c r="D38" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A38,Checklist!$D$4:$D$71,$B38,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E38" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A38,Checklist!$D$4:$D$71,$B38,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F38" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A38,Checklist!$D$4:$D$71,$B38,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G38" s="6">
-        <f>IF(C38=0,0,D38/C38)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>Affecter chauffeur à véhicule</t>
-        </is>
-      </c>
-      <c r="C39" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A39,Checklist!$D$4:$D$71,$B39)</f>
-        <v/>
-      </c>
-      <c r="D39" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A39,Checklist!$D$4:$D$71,$B39,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E39" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A39,Checklist!$D$4:$D$71,$B39,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F39" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A39,Checklist!$D$4:$D$71,$B39,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G39" s="6">
-        <f>IF(C39=0,0,D39/C39)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>Établir contrat recette ou location, avenant</t>
-        </is>
-      </c>
-      <c r="C40" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A40,Checklist!$D$4:$D$71,$B40)</f>
-        <v/>
-      </c>
-      <c r="D40" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A40,Checklist!$D$4:$D$71,$B40,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E40" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A40,Checklist!$D$4:$D$71,$B40,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F40" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A40,Checklist!$D$4:$D$71,$B40,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G40" s="6">
-        <f>IF(C40=0,0,D40/C40)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>Accorder exonération motivée / journée exceptionnelle</t>
-        </is>
-      </c>
-      <c r="C41" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A41,Checklist!$D$4:$D$71,$B41)</f>
-        <v/>
-      </c>
-      <c r="D41" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A41,Checklist!$D$4:$D$71,$B41,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E41" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A41,Checklist!$D$4:$D$71,$B41,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F41" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A41,Checklist!$D$4:$D$71,$B41,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G41" s="6">
-        <f>IF(C41=0,0,D41/C41)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>Lire planning et échéances journalières</t>
-        </is>
-      </c>
-      <c r="C42" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A42,Checklist!$D$4:$D$71,$B42)</f>
-        <v/>
-      </c>
-      <c r="D42" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A42,Checklist!$D$4:$D$71,$B42,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E42" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A42,Checklist!$D$4:$D$71,$B42,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F42" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A42,Checklist!$D$4:$D$71,$B42,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G42" s="6">
-        <f>IF(C42=0,0,D42/C42)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>Encaisser versement (espèces, mobile money, virement)</t>
-        </is>
-      </c>
-      <c r="C43" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A43,Checklist!$D$4:$D$71,$B43)</f>
-        <v/>
-      </c>
-      <c r="D43" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A43,Checklist!$D$4:$D$71,$B43,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E43" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A43,Checklist!$D$4:$D$71,$B43,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F43" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A43,Checklist!$D$4:$D$71,$B43,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G43" s="6">
-        <f>IF(C43=0,0,D43/C43)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="inlineStr">
-        <is>
-          <t>Gérer paiement partiel et anti-doublon</t>
-        </is>
-      </c>
-      <c r="C44" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A44,Checklist!$D$4:$D$71,$B44)</f>
-        <v/>
-      </c>
-      <c r="D44" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A44,Checklist!$D$4:$D$71,$B44,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E44" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A44,Checklist!$D$4:$D$71,$B44,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F44" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A44,Checklist!$D$4:$D$71,$B44,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G44" s="6">
-        <f>IF(C44=0,0,D44/C44)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="inlineStr">
-        <is>
-          <t>Émettre et imprimer reçu</t>
-        </is>
-      </c>
-      <c r="C45" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A45,Checklist!$D$4:$D$71,$B45)</f>
-        <v/>
-      </c>
-      <c r="D45" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A45,Checklist!$D$4:$D$71,$B45,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E45" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A45,Checklist!$D$4:$D$71,$B45,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F45" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A45,Checklist!$D$4:$D$71,$B45,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G45" s="6">
-        <f>IF(C45=0,0,D45/C45)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B46" s="5" t="inlineStr">
-        <is>
-          <t>Annuler un encaissement avec motif</t>
-        </is>
-      </c>
-      <c r="C46" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A46,Checklist!$D$4:$D$71,$B46)</f>
-        <v/>
-      </c>
-      <c r="D46" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A46,Checklist!$D$4:$D$71,$B46,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E46" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A46,Checklist!$D$4:$D$71,$B46,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F46" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A46,Checklist!$D$4:$D$71,$B46,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G46" s="6">
-        <f>IF(C46=0,0,D46/C46)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B47" s="5" t="inlineStr">
-        <is>
-          <t>Ouvrir / clôturer caisse, traiter écart</t>
-        </is>
-      </c>
-      <c r="C47" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A47,Checklist!$D$4:$D$71,$B47)</f>
-        <v/>
-      </c>
-      <c r="D47" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A47,Checklist!$D$4:$D$71,$B47,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E47" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A47,Checklist!$D$4:$D$71,$B47,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F47" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A47,Checklist!$D$4:$D$71,$B47,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G47" s="6">
-        <f>IF(C47=0,0,D47/C47)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>Saisir dépense avec justificatif</t>
-        </is>
-      </c>
-      <c r="C48" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A48,Checklist!$D$4:$D$71,$B48)</f>
-        <v/>
-      </c>
-      <c r="D48" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A48,Checklist!$D$4:$D$71,$B48,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E48" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A48,Checklist!$D$4:$D$71,$B48,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F48" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A48,Checklist!$D$4:$D$71,$B48,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G48" s="6">
-        <f>IF(C48=0,0,D48/C48)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>Valider dépenses au-delà du seuil, pointer banque</t>
-        </is>
-      </c>
-      <c r="C49" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A49,Checklist!$D$4:$D$71,$B49)</f>
-        <v/>
-      </c>
-      <c r="D49" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A49,Checklist!$D$4:$D$71,$B49,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E49" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A49,Checklist!$D$4:$D$71,$B49,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F49" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A49,Checklist!$D$4:$D$71,$B49,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G49" s="6">
-        <f>IF(C49=0,0,D49/C49)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="inlineStr">
-        <is>
-          <t>Passer écritures SYSCOHADA, extourne, lettrage</t>
-        </is>
-      </c>
-      <c r="C50" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A50,Checklist!$D$4:$D$71,$B50)</f>
-        <v/>
-      </c>
-      <c r="D50" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A50,Checklist!$D$4:$D$71,$B50,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E50" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A50,Checklist!$D$4:$D$71,$B50,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F50" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A50,Checklist!$D$4:$D$71,$B50,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G50" s="6">
-        <f>IF(C50=0,0,D50/C50)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B51" s="5" t="inlineStr">
-        <is>
-          <t>Clôturer période, tenir plan et comptes tiers</t>
-        </is>
-      </c>
-      <c r="C51" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A51,Checklist!$D$4:$D$71,$B51)</f>
-        <v/>
-      </c>
-      <c r="D51" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A51,Checklist!$D$4:$D$71,$B51,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E51" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A51,Checklist!$D$4:$D$71,$B51,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F51" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A51,Checklist!$D$4:$D$71,$B51,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G51" s="6">
-        <f>IF(C51=0,0,D51/C51)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B52" s="5" t="inlineStr">
-        <is>
-          <t>Éditer balance, grand livre, journaux</t>
-        </is>
-      </c>
-      <c r="C52" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A52,Checklist!$D$4:$D$71,$B52)</f>
-        <v/>
-      </c>
-      <c r="D52" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A52,Checklist!$D$4:$D$71,$B52,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E52" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A52,Checklist!$D$4:$D$71,$B52,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F52" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A52,Checklist!$D$4:$D$71,$B52,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G52" s="6">
-        <f>IF(C52=0,0,D52/C52)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B53" s="5" t="inlineStr">
-        <is>
-          <t>Planifier entretien préventif (km, jours)</t>
-        </is>
-      </c>
-      <c r="C53" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A53,Checklist!$D$4:$D$71,$B53)</f>
-        <v/>
-      </c>
-      <c r="D53" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A53,Checklist!$D$4:$D$71,$B53,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E53" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A53,Checklist!$D$4:$D$71,$B53,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F53" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A53,Checklist!$D$4:$D$71,$B53,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G53" s="6">
-        <f>IF(C53=0,0,D53/C53)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B54" s="5" t="inlineStr">
-        <is>
-          <t>Ouvrir ordre de maintenance, immobiliser, remettre en service</t>
-        </is>
-      </c>
-      <c r="C54" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A54,Checklist!$D$4:$D$71,$B54)</f>
-        <v/>
-      </c>
-      <c r="D54" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A54,Checklist!$D$4:$D$71,$B54,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E54" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A54,Checklist!$D$4:$D$71,$B54,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F54" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A54,Checklist!$D$4:$D$71,$B54,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G54" s="6">
-        <f>IF(C54=0,0,D54/C54)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B55" s="5" t="inlineStr">
-        <is>
-          <t>Gérer stock de pièces, seuils, inventaire</t>
-        </is>
-      </c>
-      <c r="C55" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A55,Checklist!$D$4:$D$71,$B55)</f>
-        <v/>
-      </c>
-      <c r="D55" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A55,Checklist!$D$4:$D$71,$B55,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E55" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A55,Checklist!$D$4:$D$71,$B55,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F55" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A55,Checklist!$D$4:$D$71,$B55,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G55" s="6">
-        <f>IF(C55=0,0,D55/C55)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B56" s="5" t="inlineStr">
-        <is>
-          <t>Utiliser l'agenda atelier</t>
-        </is>
-      </c>
-      <c r="C56" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A56,Checklist!$D$4:$D$71,$B56)</f>
-        <v/>
-      </c>
-      <c r="D56" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A56,Checklist!$D$4:$D$71,$B56,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E56" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A56,Checklist!$D$4:$D$71,$B56,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F56" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A56,Checklist!$D$4:$D$71,$B56,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G56" s="6">
-        <f>IF(C56=0,0,D56/C56)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B57" s="5" t="inlineStr">
-        <is>
-          <t>Déclarer et suivre un sinistre</t>
-        </is>
-      </c>
-      <c r="C57" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A57,Checklist!$D$4:$D$71,$B57)</f>
-        <v/>
-      </c>
-      <c r="D57" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A57,Checklist!$D$4:$D$71,$B57,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E57" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A57,Checklist!$D$4:$D$71,$B57,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F57" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A57,Checklist!$D$4:$D$71,$B57,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G57" s="6">
-        <f>IF(C57=0,0,D57/C57)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B58" s="5" t="inlineStr">
-        <is>
-          <t>Suivre position des taxis, zones, boîtiers</t>
-        </is>
-      </c>
-      <c r="C58" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A58,Checklist!$D$4:$D$71,$B58)</f>
-        <v/>
-      </c>
-      <c r="D58" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A58,Checklist!$D$4:$D$71,$B58,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E58" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A58,Checklist!$D$4:$D$71,$B58,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F58" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A58,Checklist!$D$4:$D$71,$B58,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G58" s="6">
-        <f>IF(C58=0,0,D58/C58)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B59" s="5" t="inlineStr">
-        <is>
-          <t>Traiter échéances de documents et demandes chauffeurs</t>
-        </is>
-      </c>
-      <c r="C59" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A59,Checklist!$D$4:$D$71,$B59)</f>
-        <v/>
-      </c>
-      <c r="D59" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A59,Checklist!$D$4:$D$71,$B59,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E59" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A59,Checklist!$D$4:$D$71,$B59,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F59" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A59,Checklist!$D$4:$D$71,$B59,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G59" s="6">
-        <f>IF(C59=0,0,D59/C59)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B60" s="5" t="inlineStr">
-        <is>
-          <t>Lire recouvrement, impayés, disponibilité, écarts</t>
-        </is>
-      </c>
-      <c r="C60" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A60,Checklist!$D$4:$D$71,$B60)</f>
-        <v/>
-      </c>
-      <c r="D60" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A60,Checklist!$D$4:$D$71,$B60,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E60" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A60,Checklist!$D$4:$D$71,$B60,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F60" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A60,Checklist!$D$4:$D$71,$B60,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G60" s="6">
-        <f>IF(C60=0,0,D60/C60)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B61" s="5" t="inlineStr">
-        <is>
-          <t>Se connecter et consulter reçus et véhicule</t>
-        </is>
-      </c>
-      <c r="C61" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A61,Checklist!$D$4:$D$71,$B61)</f>
-        <v/>
-      </c>
-      <c r="D61" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A61,Checklist!$D$4:$D$71,$B61,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E61" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A61,Checklist!$D$4:$D$71,$B61,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F61" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A61,Checklist!$D$4:$D$71,$B61,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G61" s="6">
-        <f>IF(C61=0,0,D61/C61)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B62" s="5" t="inlineStr">
-        <is>
-          <t>Déclarer incident avec photo, faire une demande</t>
-        </is>
-      </c>
-      <c r="C62" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A62,Checklist!$D$4:$D$71,$B62)</f>
-        <v/>
-      </c>
-      <c r="D62" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A62,Checklist!$D$4:$D$71,$B62,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E62" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A62,Checklist!$D$4:$D$71,$B62,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F62" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A62,Checklist!$D$4:$D$71,$B62,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G62" s="6">
-        <f>IF(C62=0,0,D62/C62)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B63" s="5" t="inlineStr">
-        <is>
-          <t>Verser sa recette et vérifier son solde</t>
-        </is>
-      </c>
-      <c r="C63" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A63,Checklist!$D$4:$D$71,$B63)</f>
-        <v/>
-      </c>
-      <c r="D63" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A63,Checklist!$D$4:$D$71,$B63,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E63" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A63,Checklist!$D$4:$D$71,$B63,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F63" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A63,Checklist!$D$4:$D$71,$B63,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G63" s="6">
-        <f>IF(C63=0,0,D63/C63)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B64" s="5" t="inlineStr">
-        <is>
-          <t>Régler matrice module × action</t>
-        </is>
-      </c>
-      <c r="C64" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A64,Checklist!$D$4:$D$71,$B64)</f>
-        <v/>
-      </c>
-      <c r="D64" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A64,Checklist!$D$4:$D$71,$B64,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E64" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A64,Checklist!$D$4:$D$71,$B64,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F64" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A64,Checklist!$D$4:$D$71,$B64,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G64" s="6">
-        <f>IF(C64=0,0,D64/C64)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="5" t="inlineStr">
-        <is>
-          <t>Gestion de taxi (Transport)</t>
-        </is>
-      </c>
-      <c r="B65" s="5" t="inlineStr">
-        <is>
-          <t>Sauvegarder / restaurer, lire audit</t>
-        </is>
-      </c>
-      <c r="C65" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A65,Checklist!$D$4:$D$71,$B65)</f>
-        <v/>
-      </c>
-      <c r="D65" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A65,Checklist!$D$4:$D$71,$B65,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E65" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A65,Checklist!$D$4:$D$71,$B65,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F65" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A65,Checklist!$D$4:$D$71,$B65,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G65" s="6">
-        <f>IF(C65=0,0,D65/C65)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="5" t="inlineStr">
-        <is>
-          <t>Transversal (Groupe)</t>
-        </is>
-      </c>
-      <c r="B66" s="5" t="inlineStr">
-        <is>
-          <t>Naviguer entre Distributions, Transport, Agro</t>
-        </is>
-      </c>
-      <c r="C66" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A66,Checklist!$D$4:$D$71,$B66)</f>
-        <v/>
-      </c>
-      <c r="D66" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A66,Checklist!$D$4:$D$71,$B66,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E66" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A66,Checklist!$D$4:$D$71,$B66,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F66" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A66,Checklist!$D$4:$D$71,$B66,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G66" s="6">
-        <f>IF(C66=0,0,D66/C66)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="5" t="inlineStr">
-        <is>
-          <t>Transversal (Groupe)</t>
-        </is>
-      </c>
-      <c r="B67" s="5" t="inlineStr">
-        <is>
-          <t>Lire vue consolidée (trésorerie, CA, créances)</t>
-        </is>
-      </c>
-      <c r="C67" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A67,Checklist!$D$4:$D$71,$B67)</f>
-        <v/>
-      </c>
-      <c r="D67" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A67,Checklist!$D$4:$D$71,$B67,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E67" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A67,Checklist!$D$4:$D$71,$B67,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F67" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A67,Checklist!$D$4:$D$71,$B67,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G67" s="6">
-        <f>IF(C67=0,0,D67/C67)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="5" t="inlineStr">
-        <is>
-          <t>Transversal (Groupe)</t>
-        </is>
-      </c>
-      <c r="B68" s="5" t="inlineStr">
-        <is>
-          <t>Installer l'application (PWA) et se déconnecter</t>
-        </is>
-      </c>
-      <c r="C68" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A68,Checklist!$D$4:$D$71,$B68)</f>
-        <v/>
-      </c>
-      <c r="D68" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A68,Checklist!$D$4:$D$71,$B68,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E68" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A68,Checklist!$D$4:$D$71,$B68,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F68" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A68,Checklist!$D$4:$D$71,$B68,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G68" s="6">
-        <f>IF(C68=0,0,D68/C68)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="5" t="inlineStr">
-        <is>
-          <t>Transversal (Groupe)</t>
-        </is>
-      </c>
-      <c r="B69" s="5" t="inlineStr">
-        <is>
-          <t>Changer son mot de passe, respecter règles de sécurité</t>
-        </is>
-      </c>
-      <c r="C69" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A69,Checklist!$D$4:$D$71,$B69)</f>
-        <v/>
-      </c>
-      <c r="D69" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A69,Checklist!$D$4:$D$71,$B69,Checklist!$G$4:$G$71,"Acquis")</f>
-        <v/>
-      </c>
-      <c r="E69" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A69,Checklist!$D$4:$D$71,$B69,Checklist!$G$4:$G$71,"En cours")</f>
-        <v/>
-      </c>
-      <c r="F69" s="5">
-        <f>COUNTIFS(Checklist!$B$4:$B$71,$A69,Checklist!$D$4:$D$71,$B69,Checklist!$G$4:$G$71,"Non acquis")</f>
-        <v/>
-      </c>
-      <c r="G69" s="6">
-        <f>IF(C69=0,0,D69/C69)</f>
         <v/>
       </c>
     </row>

</xml_diff>